<commit_message>
LOOP into Table items
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SalesBot\Desktop\UiPath\ApInvoiceProcessing\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SalesBot\Desktop\UiPath\Finance\ApInvoiceProcessing\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB882935-8429-453E-B1C3-A222215F02B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D4ABE3A-6975-45E1-9FF6-76CBD2A53E17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="57">
   <si>
     <t>Name</t>
   </si>
@@ -190,6 +190,12 @@
   </si>
   <si>
     <t>frmservlet.jnlp</t>
+  </si>
+  <si>
+    <t>DownloadFolderPath</t>
+  </si>
+  <si>
+    <t>C:\Users\SalesBot\Downloads</t>
   </si>
 </sst>
 </file>
@@ -681,7 +687,14 @@
         <v>54</v>
       </c>
     </row>
-    <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="12" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B12" t="s">
+        <v>56</v>
+      </c>
+    </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="15" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>